<commit_message>
Add print functionality and sample file download; enhance print styles and layout
</commit_message>
<xml_diff>
--- a/src/assets/students.xlsx
+++ b/src/assets/students.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>№</t>
   </si>
@@ -30,13 +30,49 @@
     <t>Прізвище, імя, по батькові</t>
   </si>
   <si>
-    <t>Глушко Олена Михайлівна</t>
-  </si>
-  <si>
     <t>Ураїнська мова</t>
   </si>
   <si>
     <t>Українська Література</t>
+  </si>
+  <si>
+    <t>Іваненко Іван Іванович</t>
+  </si>
+  <si>
+    <t>Математика</t>
+  </si>
+  <si>
+    <t>Іноземна мова</t>
+  </si>
+  <si>
+    <t>Історія України</t>
+  </si>
+  <si>
+    <t>Фізична культура</t>
+  </si>
+  <si>
+    <t>Технології</t>
+  </si>
+  <si>
+    <t>Біологія та екологія</t>
+  </si>
+  <si>
+    <t>Медична біологія</t>
+  </si>
+  <si>
+    <t>Основи латинської мови</t>
+  </si>
+  <si>
+    <t>Біонеорганічна біологія</t>
+  </si>
+  <si>
+    <t>Фізична та колоїдна хімія</t>
+  </si>
+  <si>
+    <t>Анатомія людини</t>
+  </si>
+  <si>
+    <t>Фізіологія</t>
   </si>
 </sst>
 </file>
@@ -87,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -100,7 +136,10 @@
       <alignment horizontal="center" textRotation="90" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -390,7 +429,7 @@
     <col min="4" max="4" width="4.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="108" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="125.4" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -398,23 +437,47 @@
         <v>2</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
+      <c r="E1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="P1" s="6" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
@@ -429,44 +492,92 @@
       <c r="D2" s="5">
         <v>9</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
+      <c r="E2" s="3">
+        <v>6</v>
+      </c>
+      <c r="F2" s="3">
+        <v>8</v>
+      </c>
+      <c r="G2" s="3">
+        <v>10</v>
+      </c>
+      <c r="H2" s="3">
+        <v>11</v>
+      </c>
+      <c r="I2" s="3">
+        <v>12</v>
+      </c>
+      <c r="J2" s="1">
+        <v>5</v>
+      </c>
+      <c r="K2" s="1">
+        <v>6</v>
+      </c>
+      <c r="L2" s="1">
+        <v>8</v>
+      </c>
+      <c r="M2" s="1">
+        <v>1</v>
+      </c>
+      <c r="N2" s="1">
+        <v>2</v>
+      </c>
+      <c r="O2" s="1">
+        <v>3</v>
+      </c>
+      <c r="P2" s="1">
+        <v>4</v>
+      </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A3" s="3">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="5">
+        <v>5</v>
+      </c>
+      <c r="C3" s="3">
+        <v>5</v>
+      </c>
+      <c r="D3" s="3">
+        <v>7</v>
+      </c>
+      <c r="E3" s="3">
+        <v>5</v>
+      </c>
+      <c r="F3" s="3">
+        <v>7</v>
+      </c>
+      <c r="G3" s="3">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3">
+        <v>5</v>
+      </c>
+      <c r="I3" s="3">
+        <v>7</v>
+      </c>
+      <c r="J3" s="1">
+        <v>11</v>
+      </c>
+      <c r="K3" s="1">
+        <v>12</v>
+      </c>
+      <c r="L3" s="1">
+        <v>11</v>
+      </c>
+      <c r="M3" s="1">
+        <v>10</v>
+      </c>
+      <c r="N3" s="1">
+        <v>9</v>
+      </c>
+      <c r="O3" s="1">
         <v>8</v>
       </c>
-      <c r="D3" s="5">
-        <v>5</v>
-      </c>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
+      <c r="P3" s="1">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>